<commit_message>
0.8.5 ground and tact polishing
+ добавил arty usage (затухание эффективности с повышением настрела)
+ добавил разделение на close и distant fire support
</commit_message>
<xml_diff>
--- a/enemy_brigade.xlsx
+++ b/enemy_brigade.xlsx
@@ -556,7 +556,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -624,7 +624,7 @@
       </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P3" t="n">
         <v>0</v>
@@ -744,7 +744,7 @@
       </c>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P5" t="n">
         <v>0</v>
@@ -796,7 +796,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M6" t="n">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P11" t="n">
         <v>0</v>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M14" t="n">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P17" t="n">
         <v>0</v>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M18" t="n">
@@ -1576,7 +1576,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M19" t="n">
@@ -1644,7 +1644,7 @@
       </c>
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P20" t="n">
         <v>0</v>
@@ -1756,7 +1756,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M22" t="n">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P22" t="n">
         <v>0</v>
@@ -1816,7 +1816,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M23" t="n">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2244,7 +2244,7 @@
       </c>
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P30" t="n">
         <v>0</v>
@@ -2424,7 +2424,7 @@
       </c>
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P33" t="n">
         <v>0</v>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -2536,7 +2536,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M35" t="n">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="N35" t="inlineStr"/>
       <c r="O35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P35" t="n">
         <v>0</v>
@@ -2596,7 +2596,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M36" t="n">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="N37" t="inlineStr"/>
       <c r="O37" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P37" t="n">
         <v>0</v>
@@ -2776,7 +2776,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>died_from_injury</t>
         </is>
       </c>
       <c r="M39" t="n">
@@ -2836,7 +2836,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M40" t="n">
@@ -2896,7 +2896,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M41" t="n">
@@ -2904,7 +2904,7 @@
       </c>
       <c r="N41" t="inlineStr"/>
       <c r="O41" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="P41" t="n">
         <v>0</v>
@@ -2956,7 +2956,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M42" t="n">
@@ -3016,7 +3016,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M43" t="n">
@@ -3076,7 +3076,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M44" t="n">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>killed</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M45" t="n">
@@ -3196,7 +3196,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M46" t="n">
@@ -3316,7 +3316,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M48" t="n">
@@ -3376,7 +3376,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M49" t="n">
@@ -3436,7 +3436,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M50" t="n">
@@ -3556,7 +3556,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M52" t="n">
@@ -3616,7 +3616,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M53" t="n">
@@ -3796,7 +3796,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M56" t="n">
@@ -3856,7 +3856,7 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M57" t="n">
@@ -3916,7 +3916,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>died_from_injury</t>
         </is>
       </c>
       <c r="M58" t="n">
@@ -3976,7 +3976,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M59" t="n">
@@ -4036,7 +4036,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M60" t="n">
@@ -4096,7 +4096,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>died_from_injury</t>
         </is>
       </c>
       <c r="M61" t="n">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M62" t="n">
@@ -4276,7 +4276,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M64" t="n">
@@ -4336,7 +4336,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M65" t="n">
@@ -4456,7 +4456,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M67" t="n">
@@ -4636,7 +4636,7 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M70" t="n">
@@ -4696,7 +4696,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M71" t="n">
@@ -4756,7 +4756,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>died_from_injury</t>
         </is>
       </c>
       <c r="M72" t="n">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M73" t="n">
@@ -4884,7 +4884,7 @@
       </c>
       <c r="N74" t="inlineStr"/>
       <c r="O74" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P74" t="n">
         <v>0</v>
@@ -4996,7 +4996,7 @@
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M76" t="n">
@@ -5184,7 +5184,7 @@
       </c>
       <c r="N79" t="inlineStr"/>
       <c r="O79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P79" t="n">
         <v>0</v>
@@ -5304,7 +5304,7 @@
       </c>
       <c r="N81" t="inlineStr"/>
       <c r="O81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P81" t="n">
         <v>0</v>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="N82" t="inlineStr"/>
       <c r="O82" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P82" t="n">
         <v>0</v>
@@ -5484,7 +5484,7 @@
       </c>
       <c r="N84" t="inlineStr"/>
       <c r="O84" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P84" t="n">
         <v>0</v>
@@ -5544,7 +5544,7 @@
       </c>
       <c r="N85" t="inlineStr"/>
       <c r="O85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P85" t="n">
         <v>0</v>
@@ -5596,7 +5596,7 @@
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M86" t="n">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="N87" t="inlineStr"/>
       <c r="O87" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P87" t="n">
         <v>0</v>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="N89" t="inlineStr"/>
       <c r="O89" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P89" t="n">
         <v>0</v>
@@ -5964,7 +5964,7 @@
       </c>
       <c r="N92" t="inlineStr"/>
       <c r="O92" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P92" t="n">
         <v>0</v>
@@ -6144,7 +6144,7 @@
       </c>
       <c r="N95" t="inlineStr"/>
       <c r="O95" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P95" t="n">
         <v>0</v>
@@ -6204,7 +6204,7 @@
       </c>
       <c r="N96" t="inlineStr"/>
       <c r="O96" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P96" t="n">
         <v>0</v>
@@ -6264,7 +6264,7 @@
       </c>
       <c r="N97" t="inlineStr"/>
       <c r="O97" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P97" t="n">
         <v>0</v>
@@ -6316,7 +6316,7 @@
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M98" t="n">
@@ -6436,7 +6436,7 @@
       </c>
       <c r="L100" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>alive</t>
         </is>
       </c>
       <c r="M100" t="n">
@@ -6744,7 +6744,7 @@
       </c>
       <c r="N105" t="inlineStr"/>
       <c r="O105" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P105" t="n">
         <v>0</v>
@@ -6864,7 +6864,7 @@
       </c>
       <c r="N107" t="inlineStr"/>
       <c r="O107" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P107" t="n">
         <v>0</v>
@@ -7036,7 +7036,7 @@
       </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M110" t="n">
@@ -7096,7 +7096,7 @@
       </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M111" t="n">
@@ -7344,7 +7344,7 @@
       </c>
       <c r="N115" t="inlineStr"/>
       <c r="O115" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P115" t="n">
         <v>0</v>
@@ -7396,7 +7396,7 @@
       </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M116" t="n">
@@ -7644,7 +7644,7 @@
       </c>
       <c r="N120" t="inlineStr"/>
       <c r="O120" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P120" t="n">
         <v>0</v>
@@ -7756,7 +7756,7 @@
       </c>
       <c r="L122" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M122" t="n">
@@ -7824,7 +7824,7 @@
       </c>
       <c r="N123" t="inlineStr"/>
       <c r="O123" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P123" t="n">
         <v>0</v>
@@ -8004,7 +8004,7 @@
       </c>
       <c r="N126" t="inlineStr"/>
       <c r="O126" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P126" t="n">
         <v>0</v>
@@ -8124,7 +8124,7 @@
       </c>
       <c r="N128" t="inlineStr"/>
       <c r="O128" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P128" t="n">
         <v>0</v>
@@ -8236,7 +8236,7 @@
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M130" t="n">
@@ -8304,7 +8304,7 @@
       </c>
       <c r="N131" t="inlineStr"/>
       <c r="O131" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P131" t="n">
         <v>0</v>
@@ -8416,7 +8416,7 @@
       </c>
       <c r="L133" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M133" t="n">
@@ -8476,7 +8476,7 @@
       </c>
       <c r="L134" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M134" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="N137" t="inlineStr"/>
       <c r="O137" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P137" t="n">
         <v>0</v>
@@ -8724,7 +8724,7 @@
       </c>
       <c r="N138" t="inlineStr"/>
       <c r="O138" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P138" t="n">
         <v>0</v>
@@ -8784,7 +8784,7 @@
       </c>
       <c r="N139" t="inlineStr"/>
       <c r="O139" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P139" t="n">
         <v>0</v>
@@ -8896,7 +8896,7 @@
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M141" t="n">
@@ -9016,7 +9016,7 @@
       </c>
       <c r="L143" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M143" t="n">
@@ -9024,7 +9024,7 @@
       </c>
       <c r="N143" t="inlineStr"/>
       <c r="O143" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P143" t="n">
         <v>0</v>
@@ -9136,7 +9136,7 @@
       </c>
       <c r="L145" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M145" t="n">
@@ -9196,7 +9196,7 @@
       </c>
       <c r="L146" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M146" t="n">
@@ -9256,7 +9256,7 @@
       </c>
       <c r="L147" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M147" t="n">
@@ -9316,7 +9316,7 @@
       </c>
       <c r="L148" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M148" t="n">
@@ -9376,7 +9376,7 @@
       </c>
       <c r="L149" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M149" t="n">
@@ -9436,7 +9436,7 @@
       </c>
       <c r="L150" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M150" t="n">
@@ -9496,7 +9496,7 @@
       </c>
       <c r="L151" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M151" t="n">
@@ -9556,7 +9556,7 @@
       </c>
       <c r="L152" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M152" t="n">
@@ -9616,7 +9616,7 @@
       </c>
       <c r="L153" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M153" t="n">
@@ -9676,7 +9676,7 @@
       </c>
       <c r="L154" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M154" t="n">
@@ -9736,7 +9736,7 @@
       </c>
       <c r="L155" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M155" t="n">
@@ -9796,7 +9796,7 @@
       </c>
       <c r="L156" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M156" t="n">
@@ -9856,7 +9856,7 @@
       </c>
       <c r="L157" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M157" t="n">
@@ -9916,7 +9916,7 @@
       </c>
       <c r="L158" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M158" t="n">
@@ -9976,7 +9976,7 @@
       </c>
       <c r="L159" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M159" t="n">
@@ -10036,7 +10036,7 @@
       </c>
       <c r="L160" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M160" t="n">
@@ -10096,7 +10096,7 @@
       </c>
       <c r="L161" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>died_from_injury</t>
         </is>
       </c>
       <c r="M161" t="n">
@@ -10156,7 +10156,7 @@
       </c>
       <c r="L162" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M162" t="n">
@@ -10216,7 +10216,7 @@
       </c>
       <c r="L163" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M163" t="n">
@@ -10276,7 +10276,7 @@
       </c>
       <c r="L164" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M164" t="n">
@@ -10336,7 +10336,7 @@
       </c>
       <c r="L165" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M165" t="n">
@@ -10396,7 +10396,7 @@
       </c>
       <c r="L166" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M166" t="n">
@@ -10456,7 +10456,7 @@
       </c>
       <c r="L167" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M167" t="n">
@@ -10516,7 +10516,7 @@
       </c>
       <c r="L168" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M168" t="n">
@@ -10576,7 +10576,7 @@
       </c>
       <c r="L169" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M169" t="n">
@@ -10636,7 +10636,7 @@
       </c>
       <c r="L170" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>died_from_injury</t>
         </is>
       </c>
       <c r="M170" t="n">
@@ -10696,7 +10696,7 @@
       </c>
       <c r="L171" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M171" t="n">
@@ -10704,7 +10704,7 @@
       </c>
       <c r="N171" t="inlineStr"/>
       <c r="O171" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P171" t="n">
         <v>0</v>
@@ -10756,7 +10756,7 @@
       </c>
       <c r="L172" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M172" t="n">
@@ -10816,7 +10816,7 @@
       </c>
       <c r="L173" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M173" t="n">
@@ -10876,7 +10876,7 @@
       </c>
       <c r="L174" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M174" t="n">
@@ -10936,7 +10936,7 @@
       </c>
       <c r="L175" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M175" t="n">
@@ -10996,7 +10996,7 @@
       </c>
       <c r="L176" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M176" t="n">
@@ -11056,7 +11056,7 @@
       </c>
       <c r="L177" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M177" t="n">
@@ -11116,7 +11116,7 @@
       </c>
       <c r="L178" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>died_from_injury</t>
         </is>
       </c>
       <c r="M178" t="n">
@@ -11176,7 +11176,7 @@
       </c>
       <c r="L179" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M179" t="n">
@@ -11236,7 +11236,7 @@
       </c>
       <c r="L180" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M180" t="n">
@@ -11296,7 +11296,7 @@
       </c>
       <c r="L181" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M181" t="n">
@@ -11356,7 +11356,7 @@
       </c>
       <c r="L182" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>died_from_injury</t>
         </is>
       </c>
       <c r="M182" t="n">
@@ -11416,7 +11416,7 @@
       </c>
       <c r="L183" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M183" t="n">
@@ -11476,7 +11476,7 @@
       </c>
       <c r="L184" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M184" t="n">
@@ -11536,7 +11536,7 @@
       </c>
       <c r="L185" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M185" t="n">
@@ -11724,7 +11724,7 @@
       </c>
       <c r="N188" t="inlineStr"/>
       <c r="O188" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P188" t="n">
         <v>0</v>
@@ -11776,7 +11776,7 @@
       </c>
       <c r="L189" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M189" t="n">
@@ -11836,7 +11836,7 @@
       </c>
       <c r="L190" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M190" t="n">
@@ -11956,7 +11956,7 @@
       </c>
       <c r="L192" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M192" t="n">
@@ -12084,7 +12084,7 @@
       </c>
       <c r="N194" t="inlineStr"/>
       <c r="O194" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P194" t="n">
         <v>0</v>
@@ -12136,7 +12136,7 @@
       </c>
       <c r="L195" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M195" t="n">
@@ -12144,7 +12144,7 @@
       </c>
       <c r="N195" t="inlineStr"/>
       <c r="O195" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P195" t="n">
         <v>0</v>
@@ -12204,7 +12204,7 @@
       </c>
       <c r="N196" t="inlineStr"/>
       <c r="O196" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P196" t="n">
         <v>0</v>
@@ -12264,7 +12264,7 @@
       </c>
       <c r="N197" t="inlineStr"/>
       <c r="O197" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P197" t="n">
         <v>0</v>
@@ -12564,7 +12564,7 @@
       </c>
       <c r="N202" t="inlineStr"/>
       <c r="O202" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P202" t="n">
         <v>0</v>
@@ -12616,7 +12616,7 @@
       </c>
       <c r="L203" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M203" t="n">
@@ -12684,7 +12684,7 @@
       </c>
       <c r="N204" t="inlineStr"/>
       <c r="O204" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P204" t="n">
         <v>0</v>
@@ -12744,7 +12744,7 @@
       </c>
       <c r="N205" t="inlineStr"/>
       <c r="O205" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P205" t="n">
         <v>0</v>
@@ -12856,7 +12856,7 @@
       </c>
       <c r="L207" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>died_from_injury</t>
         </is>
       </c>
       <c r="M207" t="n">
@@ -12864,7 +12864,7 @@
       </c>
       <c r="N207" t="inlineStr"/>
       <c r="O207" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P207" t="n">
         <v>0</v>
@@ -13104,7 +13104,7 @@
       </c>
       <c r="N211" t="inlineStr"/>
       <c r="O211" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P211" t="n">
         <v>0</v>
@@ -13164,7 +13164,7 @@
       </c>
       <c r="N212" t="inlineStr"/>
       <c r="O212" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P212" t="n">
         <v>0</v>
@@ -13284,7 +13284,7 @@
       </c>
       <c r="N214" t="inlineStr"/>
       <c r="O214" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P214" t="n">
         <v>0</v>
@@ -13516,7 +13516,7 @@
       </c>
       <c r="L218" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M218" t="n">
@@ -13576,7 +13576,7 @@
       </c>
       <c r="L219" t="inlineStr">
         <is>
-          <t>killed</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M219" t="n">
@@ -13636,7 +13636,7 @@
       </c>
       <c r="L220" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M220" t="n">
@@ -13696,7 +13696,7 @@
       </c>
       <c r="L221" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M221" t="n">
@@ -13756,7 +13756,7 @@
       </c>
       <c r="L222" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M222" t="n">
@@ -13816,7 +13816,7 @@
       </c>
       <c r="L223" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M223" t="n">
@@ -13876,7 +13876,7 @@
       </c>
       <c r="L224" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M224" t="n">
@@ -13884,7 +13884,7 @@
       </c>
       <c r="N224" t="inlineStr"/>
       <c r="O224" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P224" t="n">
         <v>0</v>
@@ -13936,7 +13936,7 @@
       </c>
       <c r="L225" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M225" t="n">
@@ -13996,7 +13996,7 @@
       </c>
       <c r="L226" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M226" t="n">
@@ -14056,7 +14056,7 @@
       </c>
       <c r="L227" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>died_from_injury</t>
         </is>
       </c>
       <c r="M227" t="n">
@@ -14116,7 +14116,7 @@
       </c>
       <c r="L228" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M228" t="n">
@@ -14176,7 +14176,7 @@
       </c>
       <c r="L229" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>died_from_injury</t>
         </is>
       </c>
       <c r="M229" t="n">
@@ -14236,7 +14236,7 @@
       </c>
       <c r="L230" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M230" t="n">
@@ -14296,7 +14296,7 @@
       </c>
       <c r="L231" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M231" t="n">
@@ -14356,7 +14356,7 @@
       </c>
       <c r="L232" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M232" t="n">
@@ -14416,7 +14416,7 @@
       </c>
       <c r="L233" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M233" t="n">
@@ -14476,7 +14476,7 @@
       </c>
       <c r="L234" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M234" t="n">
@@ -14536,7 +14536,7 @@
       </c>
       <c r="L235" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M235" t="n">
@@ -14596,7 +14596,7 @@
       </c>
       <c r="L236" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M236" t="n">
@@ -14656,7 +14656,7 @@
       </c>
       <c r="L237" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M237" t="n">
@@ -14716,7 +14716,7 @@
       </c>
       <c r="L238" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M238" t="n">
@@ -14896,7 +14896,7 @@
       </c>
       <c r="L241" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M241" t="n">
@@ -14904,7 +14904,7 @@
       </c>
       <c r="N241" t="inlineStr"/>
       <c r="O241" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P241" t="n">
         <v>0</v>
@@ -14956,7 +14956,7 @@
       </c>
       <c r="L242" t="inlineStr">
         <is>
-          <t>died_from_injury</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M242" t="n">
@@ -15076,7 +15076,7 @@
       </c>
       <c r="L244" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M244" t="n">
@@ -15136,7 +15136,7 @@
       </c>
       <c r="L245" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M245" t="n">
@@ -15196,7 +15196,7 @@
       </c>
       <c r="L246" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M246" t="n">
@@ -15256,7 +15256,7 @@
       </c>
       <c r="L247" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M247" t="n">
@@ -15316,7 +15316,7 @@
       </c>
       <c r="L248" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M248" t="n">
@@ -15436,7 +15436,7 @@
       </c>
       <c r="L250" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M250" t="n">
@@ -15616,7 +15616,7 @@
       </c>
       <c r="L253" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>died_from_injury</t>
         </is>
       </c>
       <c r="M253" t="n">
@@ -15676,7 +15676,7 @@
       </c>
       <c r="L254" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M254" t="n">
@@ -15736,7 +15736,7 @@
       </c>
       <c r="L255" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M255" t="n">
@@ -15796,7 +15796,7 @@
       </c>
       <c r="L256" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M256" t="n">
@@ -15856,7 +15856,7 @@
       </c>
       <c r="L257" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M257" t="n">
@@ -15916,7 +15916,7 @@
       </c>
       <c r="L258" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M258" t="n">
@@ -15976,7 +15976,7 @@
       </c>
       <c r="L259" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M259" t="n">
@@ -16036,7 +16036,7 @@
       </c>
       <c r="L260" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M260" t="n">
@@ -16096,7 +16096,7 @@
       </c>
       <c r="L261" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M261" t="n">
@@ -16156,7 +16156,7 @@
       </c>
       <c r="L262" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M262" t="n">
@@ -16216,7 +16216,7 @@
       </c>
       <c r="L263" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M263" t="n">
@@ -16276,7 +16276,7 @@
       </c>
       <c r="L264" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M264" t="n">
@@ -16336,7 +16336,7 @@
       </c>
       <c r="L265" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M265" t="n">
@@ -16396,7 +16396,7 @@
       </c>
       <c r="L266" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M266" t="n">
@@ -16456,7 +16456,7 @@
       </c>
       <c r="L267" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>died_from_injury</t>
         </is>
       </c>
       <c r="M267" t="n">
@@ -16516,7 +16516,7 @@
       </c>
       <c r="L268" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M268" t="n">
@@ -16576,7 +16576,7 @@
       </c>
       <c r="L269" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M269" t="n">
@@ -16636,7 +16636,7 @@
       </c>
       <c r="L270" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M270" t="n">
@@ -16644,7 +16644,7 @@
       </c>
       <c r="N270" t="inlineStr"/>
       <c r="O270" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P270" t="n">
         <v>0</v>
@@ -16696,7 +16696,7 @@
       </c>
       <c r="L271" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M271" t="n">
@@ -16756,7 +16756,7 @@
       </c>
       <c r="L272" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M272" t="n">
@@ -16816,7 +16816,7 @@
       </c>
       <c r="L273" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M273" t="n">
@@ -16876,7 +16876,7 @@
       </c>
       <c r="L274" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M274" t="n">
@@ -16936,7 +16936,7 @@
       </c>
       <c r="L275" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M275" t="n">
@@ -16996,7 +16996,7 @@
       </c>
       <c r="L276" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M276" t="n">
@@ -17056,7 +17056,7 @@
       </c>
       <c r="L277" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M277" t="n">
@@ -17116,7 +17116,7 @@
       </c>
       <c r="L278" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M278" t="n">
@@ -17176,7 +17176,7 @@
       </c>
       <c r="L279" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M279" t="n">
@@ -17236,7 +17236,7 @@
       </c>
       <c r="L280" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M280" t="n">
@@ -17244,7 +17244,7 @@
       </c>
       <c r="N280" t="inlineStr"/>
       <c r="O280" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P280" t="n">
         <v>0</v>
@@ -17296,7 +17296,7 @@
       </c>
       <c r="L281" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M281" t="n">
@@ -17356,7 +17356,7 @@
       </c>
       <c r="L282" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M282" t="n">
@@ -17416,7 +17416,7 @@
       </c>
       <c r="L283" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M283" t="n">
@@ -17476,7 +17476,7 @@
       </c>
       <c r="L284" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M284" t="n">
@@ -17536,7 +17536,7 @@
       </c>
       <c r="L285" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M285" t="n">
@@ -17596,7 +17596,7 @@
       </c>
       <c r="L286" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M286" t="n">
@@ -17656,7 +17656,7 @@
       </c>
       <c r="L287" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M287" t="n">
@@ -17716,7 +17716,7 @@
       </c>
       <c r="L288" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M288" t="n">
@@ -17776,7 +17776,7 @@
       </c>
       <c r="L289" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M289" t="n">
@@ -17836,7 +17836,7 @@
       </c>
       <c r="L290" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>died_from_injury</t>
         </is>
       </c>
       <c r="M290" t="n">
@@ -17956,7 +17956,7 @@
       </c>
       <c r="L292" t="inlineStr">
         <is>
-          <t>killed</t>
+          <t>died_from_injury</t>
         </is>
       </c>
       <c r="M292" t="n">
@@ -18016,7 +18016,7 @@
       </c>
       <c r="L293" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M293" t="n">
@@ -18076,7 +18076,7 @@
       </c>
       <c r="L294" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M294" t="n">
@@ -18196,7 +18196,7 @@
       </c>
       <c r="L296" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M296" t="n">
@@ -18256,7 +18256,7 @@
       </c>
       <c r="L297" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M297" t="n">
@@ -18316,7 +18316,7 @@
       </c>
       <c r="L298" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M298" t="n">
@@ -18376,7 +18376,7 @@
       </c>
       <c r="L299" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M299" t="n">
@@ -18436,7 +18436,7 @@
       </c>
       <c r="L300" t="inlineStr">
         <is>
-          <t>killed</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M300" t="n">
@@ -18496,7 +18496,7 @@
       </c>
       <c r="L301" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M301" t="n">
@@ -18556,7 +18556,7 @@
       </c>
       <c r="L302" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M302" t="n">
@@ -18676,7 +18676,7 @@
       </c>
       <c r="L304" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M304" t="n">
@@ -18736,7 +18736,7 @@
       </c>
       <c r="L305" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M305" t="n">
@@ -18744,7 +18744,7 @@
       </c>
       <c r="N305" t="inlineStr"/>
       <c r="O305" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P305" t="n">
         <v>0</v>
@@ -18796,7 +18796,7 @@
       </c>
       <c r="L306" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>died_from_injury</t>
         </is>
       </c>
       <c r="M306" t="n">
@@ -18856,7 +18856,7 @@
       </c>
       <c r="L307" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M307" t="n">
@@ -18916,7 +18916,7 @@
       </c>
       <c r="L308" t="inlineStr">
         <is>
-          <t>heavy</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M308" t="n">
@@ -18976,7 +18976,7 @@
       </c>
       <c r="L309" t="inlineStr">
         <is>
-          <t>killed</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M309" t="n">
@@ -19036,7 +19036,7 @@
       </c>
       <c r="L310" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M310" t="n">
@@ -19276,7 +19276,7 @@
       </c>
       <c r="L314" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>light</t>
         </is>
       </c>
       <c r="M314" t="n">
@@ -19336,7 +19336,7 @@
       </c>
       <c r="L315" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M315" t="n">
@@ -19456,7 +19456,7 @@
       </c>
       <c r="L317" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M317" t="n">
@@ -19576,7 +19576,7 @@
       </c>
       <c r="L319" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M319" t="n">
@@ -19584,7 +19584,7 @@
       </c>
       <c r="N319" t="inlineStr"/>
       <c r="O319" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P319" t="n">
         <v>0</v>
@@ -19756,7 +19756,7 @@
       </c>
       <c r="L322" t="inlineStr">
         <is>
-          <t>alive</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M322" t="n">
@@ -19816,7 +19816,7 @@
       </c>
       <c r="L323" t="inlineStr">
         <is>
-          <t>light</t>
+          <t>heavy</t>
         </is>
       </c>
       <c r="M323" t="n">
@@ -19876,7 +19876,7 @@
       </c>
       <c r="L324" t="inlineStr">
         <is>
-          <t>died_from_injury</t>
+          <t>killed</t>
         </is>
       </c>
       <c r="M324" t="n">
@@ -19944,7 +19944,7 @@
       </c>
       <c r="N325" t="inlineStr"/>
       <c r="O325" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P325" t="n">
         <v>0</v>

</xml_diff>